<commit_message>
Update dashboard: honest titles, one-decimal labels, 8th of 19 card
</commit_message>
<xml_diff>
--- a/CQC_dashboard.xlsx
+++ b/CQC_dashboard.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ecoin\Downloads\CQC_SQL_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{344A9A50-43A7-45A7-8FC4-F5A730DB5BC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{233D0490-616B-45B4-B0F1-E01B3A9CD276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6063B72E-662F-42A3-B801-4B9188A9453D}"/>
   </bookViews>
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -129,7 +129,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="228">
   <si>
     <t>region</t>
   </si>
@@ -810,6 +810,9 @@
   </si>
   <si>
     <t>Source: CQC care directory with ratings, 1 Oct 2026 release (public data). 13,448 rated care homes in England. Analysis: Raphael Akhigbe (PostgreSQL + Excel).</t>
+  </si>
+  <si>
+    <t>8th of 19 in South East</t>
   </si>
 </sst>
 </file>
@@ -1098,7 +1101,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1112,7 +1115,6 @@
     <xf numFmtId="164" fontId="2" fillId="3" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1120,7 +1122,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
@@ -1128,7 +1129,7 @@
     <xf numFmtId="165" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1164,18 +1165,6 @@
   <dxfs count="17">
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -1193,6 +1182,18 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1280,45 +1281,9 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-GB" sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:sysClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:rPr>
-              <a:t>West Sussex mirrors England: 8 in 10 homes Good, and no Inadequate homes locally</a:t>
+              <a:rPr lang="en-GB" sz="1400" b="1" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t>West Sussex is in line with England: about 8 in 10 homes Good, none Inadequate locally</a:t>
             </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr algn="ctr" rtl="0">
-              <a:defRPr lang="en-GB" sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:sysClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-GB" sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:sysClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:endParaRPr>
           </a:p>
         </c:rich>
       </c:tx>
@@ -1383,6 +1348,7 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:numFmt formatCode="0.0" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -1512,6 +1478,7 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:numFmt formatCode="0.0" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -1855,34 +1822,9 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-GB" sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:sysClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:rPr>
-              <a:t>West Sussex beats England in both home types, with its biggest lead in nursing homes</a:t>
+              <a:rPr lang="en-GB" sz="1400" b="1" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t>Nursing homes rate lower nationally; West Sussex is similar to England in both types</a:t>
             </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr algn="ctr" rtl="0">
-              <a:defRPr lang="en-GB" sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:sysClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
             <a:endParaRPr lang="en-GB" sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
                 <a:sysClr val="windowText" lastClr="000000">
@@ -1958,6 +1900,7 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:numFmt formatCode="0.0" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -2289,6 +2232,7 @@
         <c:crossAx val="1438747007"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="20"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -2474,6 +2418,7 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:numFmt formatCode="0.0" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -2787,19 +2732,20 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-GB" sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:sysClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:rPr>
-              <a:t>West Sussex dementia homes outperform England’s, while its non-dementia homes trail behind</a:t>
+              <a:rPr lang="en-GB" sz="1400" b="1" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t>Dementia homes rate 6.8 points lower nationally; West Sussex's don't follow that pattern (small numbers)</a:t>
             </a:r>
+            <a:endParaRPr lang="en-GB" sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:endParaRPr>
           </a:p>
         </c:rich>
       </c:tx>
@@ -4162,6 +4108,7 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:numFmt formatCode="0.0" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -8501,12 +8448,12 @@
   </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>581396</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>128716</xdr:colOff>
       <xdr:row>89</xdr:row>
       <xdr:rowOff>12371</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="18038443" cy="4168734"/>
+    <xdr:ext cx="17886157" cy="3849116"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="9" name="TextBox 8">
@@ -8520,8 +8467,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="581396" y="19784427"/>
-          <a:ext cx="18038443" cy="4168734"/>
+          <a:off x="733682" y="18985141"/>
+          <a:ext cx="17886157" cy="3849116"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8548,58 +8495,559 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr lvl="0" rtl="0"/>
+          <a:pPr lvl="0"/>
           <a:r>
-            <a:rPr lang="en-GB" sz="2000" b="0" i="1"/>
-            <a:t>1. West Sussex: 84.1% of rated homes are Good or Outstanding, slightly above England (82.6%) and the South East (81.9%).</a:t>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>1.</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Old ratings may overstate today's quality:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>72.9%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> of ratings are over 2 years old, and recent ratings are far lower (</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>70.8%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> vs </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>87.0%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> Good or Outstanding). CQC re-inspects weaker homes sooner, and introduced a new assessment framework from late 2023, so part of the gap may reflect the change in method.</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr lvl="0" rtl="0"/>
-          <a:endParaRPr lang="en-GB" sz="2000" b="0"/>
-        </a:p>
-        <a:p>
-          <a:pPr lvl="0" rtl="0"/>
+          <a:pPr lvl="0"/>
           <a:r>
-            <a:rPr lang="en-GB" sz="2000" b="0" i="1"/>
-            <a:t>2. West Sussex is 2.2 points above the South East average, 51st of 140 authorities when each is compared with its own region.</a:t>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>2. Leadership and safety drive poor ratings:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> of the </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>2,342</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> homes rated below Good, </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>98.2%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> fall short on Well-led and </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>93.1%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> on Safe, but only </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>21.9%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> on Caring.</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr lvl="0" rtl="0"/>
-          <a:endParaRPr lang="en-GB" sz="2000" b="0"/>
-        </a:p>
-        <a:p>
-          <a:pPr lvl="0" rtl="0"/>
+          <a:pPr lvl="0"/>
           <a:r>
-            <a:rPr lang="en-GB" sz="2000" b="0" i="1"/>
-            <a:t>3. Nationally, homes run by larger providers rate higher (79.0% for single-home owners to 87.3% for groups of 21+), possibly reflecting shared systems. West Sussex dementia homes (84.8%) beat England’s (79.6%).</a:t>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>3. Dementia homes rate lower nationally:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>79.6%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> Good or Outstanding vs </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>86.4%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> for other homes.</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr lvl="0" rtl="0"/>
-          <a:endParaRPr lang="en-GB" sz="2000" b="0" i="1"/>
-        </a:p>
-        <a:p>
-          <a:pPr lvl="0" rtl="0"/>
+          <a:pPr lvl="0"/>
           <a:r>
-            <a:rPr lang="en-GB" sz="2000" b="0" i="1"/>
-            <a:t>4. Of the 2,342 homes rated below Good, over 9 in 10 fall short on Well-led (98.2%) and Safe (93.1%), but only about 1 in 5 on Caring (21.9%).</a:t>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>4. Larger providers rate higher:</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> from </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>79.0%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> for single-home owners to </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>87.3%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> for groups of 21+ homes. This is a correlation; the data cannot show why.</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr lvl="0" rtl="0"/>
-          <a:endParaRPr lang="en-GB" sz="2000" b="0"/>
-        </a:p>
-        <a:p>
-          <a:pPr lvl="0" rtl="0"/>
+          <a:pPr lvl="0"/>
           <a:r>
-            <a:rPr lang="en-GB" sz="2000" b="1" i="1"/>
-            <a:t>Caution: 72.9% of ratings are over 2 years old, and recent inspections rate fewer homes Good (70.8% vs 87.0%). Small homes’ high scores may reflect their learning-disability focus, not their size.</a:t>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>5. West Sussex is in line with England:</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-GB" sz="1100"/>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>84.1%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> vs </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>82.6%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>, a gap within the roughly ±4-point margin for 315 homes. It ranks </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>69th of 140</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> authorities nationally and </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>8th of 19</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2400" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> in the </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2000" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>South East. Its dementia homes (</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2000" b="1" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>84.8%</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="2000" b="0" i="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>) do not show the national dip, but with 165 homes treat that with care.</a:t>
+          </a:r>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -9259,7 +9707,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" ht="66" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="18" t="s">
         <v>203</v>
       </c>
     </row>
@@ -9293,7 +9741,7 @@
         <f>_xlfn.XLOOKUP("South East", q2c_region_rank[region], q2c_region_rank[pct_good_or_outstanding])</f>
         <v>81.900000000000006</v>
       </c>
-      <c r="H3" s="18">
+      <c r="H3" s="16">
         <f>_xlfn.XLOOKUP("west sussex",q9_la_vs_region[local_authority],q9_la_vs_region[gap])</f>
         <v>2.2000000000000002</v>
       </c>
@@ -9302,58 +9750,57 @@
         <v>72.900000000000006</v>
       </c>
     </row>
-    <row r="4" spans="2:10" s="25" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B4" s="24">
+    <row r="4" spans="2:10" s="23" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B4" s="22">
         <f>_xlfn.XLOOKUP("England", q1_good_or_outstanding[area], q1_good_or_outstanding[rated_homes])</f>
         <v>13448</v>
       </c>
-      <c r="D4" s="26">
+      <c r="D4" s="24">
         <f>_xlfn.XLOOKUP("west sussex", q1_good_or_outstanding[area], q1_good_or_outstanding[rated_homes])</f>
         <v>315</v>
       </c>
-      <c r="F4" s="24">
+      <c r="F4" s="22">
         <f>_xlfn.XLOOKUP("South East", q2c_region_rank[region], q2c_region_rank[rated_homes])</f>
         <v>2530</v>
       </c>
-      <c r="H4" s="27">
-        <f>_xlfn.XMATCH("west sussex",q9_la_vs_region[local_authority])</f>
-        <v>51</v>
-      </c>
-      <c r="J4" s="28" cm="1">
+      <c r="H4" s="25" t="s">
+        <v>227</v>
+      </c>
+      <c r="J4" s="26" cm="1">
         <f t="array" ref="J4">q8_rating_age_step_1[older_than_2y]</f>
         <v>9809</v>
       </c>
     </row>
     <row r="57" spans="7:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="G57" s="8" t="s">
+      <c r="G57" s="7" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="59" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G59" s="6" t="s">
+      <c r="G59" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="H59" s="6" t="s">
+      <c r="H59" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="61" spans="7:12" x14ac:dyDescent="0.25">
-      <c r="G61" s="29" t="s">
+      <c r="G61" s="27" t="s">
         <v>218</v>
       </c>
-      <c r="H61" s="30" t="s">
+      <c r="H61" s="28" t="s">
         <v>219</v>
       </c>
-      <c r="I61" s="22" t="s">
+      <c r="I61" s="20" t="s">
         <v>220</v>
       </c>
-      <c r="J61" s="22" t="s">
+      <c r="J61" s="20" t="s">
         <v>221</v>
       </c>
-      <c r="K61" s="22" t="s">
+      <c r="K61" s="20" t="s">
         <v>222</v>
       </c>
-      <c r="L61" s="23" t="s">
+      <c r="L61" s="21" t="s">
         <v>223</v>
       </c>
     </row>
@@ -9374,7 +9821,7 @@
       <c r="K62">
         <v>81.900000000000006</v>
       </c>
-      <c r="L62" s="7">
+      <c r="L62" s="6">
         <v>11</v>
       </c>
     </row>
@@ -9394,7 +9841,7 @@
       <c r="K63">
         <v>81.900000000000006</v>
       </c>
-      <c r="L63" s="7">
+      <c r="L63" s="6">
         <v>9.6</v>
       </c>
     </row>
@@ -9414,7 +9861,7 @@
       <c r="K64">
         <v>81.900000000000006</v>
       </c>
-      <c r="L64" s="7">
+      <c r="L64" s="6">
         <v>7.8</v>
       </c>
     </row>
@@ -9434,7 +9881,7 @@
       <c r="K65">
         <v>81.900000000000006</v>
       </c>
-      <c r="L65" s="7">
+      <c r="L65" s="6">
         <v>6.2</v>
       </c>
     </row>
@@ -9454,7 +9901,7 @@
       <c r="K66">
         <v>81.900000000000006</v>
       </c>
-      <c r="L66" s="7">
+      <c r="L66" s="6">
         <v>5.8</v>
       </c>
     </row>
@@ -9474,7 +9921,7 @@
       <c r="K67">
         <v>81.900000000000006</v>
       </c>
-      <c r="L67" s="7">
+      <c r="L67" s="6">
         <v>3</v>
       </c>
     </row>
@@ -9494,7 +9941,7 @@
       <c r="K68">
         <v>81.900000000000006</v>
       </c>
-      <c r="L68" s="7">
+      <c r="L68" s="6">
         <v>2.7</v>
       </c>
     </row>
@@ -9514,7 +9961,7 @@
       <c r="K69">
         <v>81.900000000000006</v>
       </c>
-      <c r="L69" s="7">
+      <c r="L69" s="6">
         <v>2.2000000000000002</v>
       </c>
     </row>
@@ -9534,7 +9981,7 @@
       <c r="K70">
         <v>81.900000000000006</v>
       </c>
-      <c r="L70" s="7">
+      <c r="L70" s="6">
         <v>1.1000000000000001</v>
       </c>
     </row>
@@ -9554,7 +10001,7 @@
       <c r="K71">
         <v>81.900000000000006</v>
       </c>
-      <c r="L71" s="7">
+      <c r="L71" s="6">
         <v>-0.6</v>
       </c>
     </row>
@@ -9574,7 +10021,7 @@
       <c r="K72">
         <v>81.900000000000006</v>
       </c>
-      <c r="L72" s="7">
+      <c r="L72" s="6">
         <v>-3</v>
       </c>
     </row>
@@ -9594,7 +10041,7 @@
       <c r="K73">
         <v>81.900000000000006</v>
       </c>
-      <c r="L73" s="7">
+      <c r="L73" s="6">
         <v>-6</v>
       </c>
     </row>
@@ -9614,7 +10061,7 @@
       <c r="K74">
         <v>81.900000000000006</v>
       </c>
-      <c r="L74" s="7">
+      <c r="L74" s="6">
         <v>-9.5</v>
       </c>
     </row>
@@ -9634,7 +10081,7 @@
       <c r="K75">
         <v>81.900000000000006</v>
       </c>
-      <c r="L75" s="7">
+      <c r="L75" s="6">
         <v>-10</v>
       </c>
     </row>
@@ -9654,7 +10101,7 @@
       <c r="K76">
         <v>81.900000000000006</v>
       </c>
-      <c r="L76" s="7">
+      <c r="L76" s="6">
         <v>-10.5</v>
       </c>
     </row>
@@ -9674,7 +10121,7 @@
       <c r="K77">
         <v>81.900000000000006</v>
       </c>
-      <c r="L77" s="7">
+      <c r="L77" s="6">
         <v>-10.7</v>
       </c>
     </row>
@@ -9694,370 +10141,138 @@
       <c r="K78">
         <v>81.900000000000006</v>
       </c>
-      <c r="L78" s="7">
+      <c r="L78" s="6">
         <v>-11.9</v>
       </c>
     </row>
-    <row r="82" spans="2:12" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="B82" s="19"/>
-      <c r="C82" s="13"/>
-      <c r="D82" s="13"/>
-      <c r="E82" s="13"/>
-      <c r="G82" s="13"/>
-      <c r="H82" s="13"/>
-      <c r="I82" s="13"/>
-      <c r="J82" s="13"/>
-      <c r="K82" s="13"/>
-      <c r="L82" s="13"/>
-    </row>
-    <row r="83" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B83" s="13"/>
-      <c r="C83" s="13"/>
-      <c r="D83" s="13"/>
-      <c r="E83" s="13"/>
-      <c r="G83" s="13"/>
-      <c r="H83" s="13"/>
-      <c r="I83" s="13"/>
-      <c r="J83" s="13"/>
-      <c r="K83" s="13"/>
-      <c r="L83" s="13"/>
-    </row>
-    <row r="84" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B84" s="13"/>
-      <c r="C84" s="13"/>
-      <c r="D84" s="13"/>
-      <c r="E84" s="13"/>
-      <c r="G84" s="13"/>
-      <c r="H84" s="13"/>
-      <c r="I84" s="13"/>
-      <c r="J84" s="13"/>
-      <c r="K84" s="13"/>
-      <c r="L84" s="13"/>
-    </row>
-    <row r="85" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B85" s="13"/>
-      <c r="C85" s="13"/>
-      <c r="D85" s="13"/>
-      <c r="E85" s="13"/>
-      <c r="G85" s="13"/>
-      <c r="H85" s="13"/>
-      <c r="I85" s="13"/>
-      <c r="J85" s="13"/>
-      <c r="K85" s="13"/>
-      <c r="L85" s="13"/>
-    </row>
-    <row r="86" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B86" s="13"/>
-      <c r="C86" s="13"/>
-      <c r="D86" s="13"/>
-      <c r="E86" s="13"/>
-      <c r="G86" s="13"/>
-      <c r="H86" s="13"/>
-      <c r="I86" s="13"/>
-      <c r="J86" s="13"/>
-      <c r="K86" s="13"/>
-      <c r="L86" s="13"/>
-    </row>
-    <row r="87" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B87" s="13"/>
-      <c r="C87" s="13"/>
-      <c r="D87" s="13"/>
-      <c r="E87" s="13"/>
-      <c r="G87" s="13"/>
-      <c r="H87" s="13"/>
-      <c r="I87" s="13"/>
-      <c r="J87" s="13"/>
-      <c r="K87" s="13"/>
-      <c r="L87" s="13"/>
-    </row>
-    <row r="88" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B88" s="13"/>
-      <c r="C88" s="13"/>
-      <c r="D88" s="13"/>
-      <c r="E88" s="13"/>
-      <c r="G88" s="13"/>
-      <c r="H88" s="13"/>
-      <c r="I88" s="13"/>
-      <c r="J88" s="13"/>
-      <c r="K88" s="13"/>
-      <c r="L88" s="13"/>
-    </row>
-    <row r="89" spans="2:12" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="B89" s="9" t="s">
+    <row r="82" spans="2:11" ht="31.5" x14ac:dyDescent="0.5">
+      <c r="B82" s="17"/>
+    </row>
+    <row r="88" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="89" spans="2:11" ht="31.5" x14ac:dyDescent="0.5">
+      <c r="B89" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="C89" s="10"/>
-      <c r="D89" s="10"/>
-      <c r="E89" s="10"/>
-      <c r="F89" s="10"/>
-      <c r="G89" s="10"/>
-      <c r="H89" s="10"/>
-      <c r="I89" s="10"/>
-      <c r="J89" s="10"/>
-      <c r="K89" s="11"/>
-    </row>
-    <row r="90" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B90" s="12"/>
-      <c r="C90" s="13"/>
-      <c r="D90" s="13"/>
-      <c r="E90" s="13"/>
-      <c r="F90" s="13"/>
-      <c r="G90" s="13"/>
-      <c r="H90" s="13"/>
-      <c r="I90" s="13"/>
-      <c r="J90" s="13"/>
-      <c r="K90" s="14"/>
-    </row>
-    <row r="91" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B91" s="12"/>
-      <c r="C91" s="13"/>
-      <c r="D91" s="13"/>
-      <c r="E91" s="13"/>
-      <c r="F91" s="13"/>
-      <c r="G91" s="13"/>
-      <c r="H91" s="13"/>
-      <c r="I91" s="13"/>
-      <c r="J91" s="13"/>
-      <c r="K91" s="14"/>
-    </row>
-    <row r="92" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B92" s="12"/>
-      <c r="C92" s="13"/>
-      <c r="D92" s="13"/>
-      <c r="E92" s="13"/>
-      <c r="F92" s="13"/>
-      <c r="G92" s="13"/>
-      <c r="H92" s="13"/>
-      <c r="I92" s="13"/>
-      <c r="J92" s="13"/>
-      <c r="K92" s="14"/>
-    </row>
-    <row r="93" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B93" s="12"/>
-      <c r="C93" s="13"/>
-      <c r="D93" s="13"/>
-      <c r="E93" s="13"/>
-      <c r="F93" s="13"/>
-      <c r="G93" s="13"/>
-      <c r="H93" s="13"/>
-      <c r="I93" s="13"/>
-      <c r="J93" s="13"/>
-      <c r="K93" s="14"/>
-    </row>
-    <row r="94" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B94" s="12"/>
-      <c r="C94" s="13"/>
-      <c r="D94" s="13"/>
-      <c r="E94" s="13"/>
-      <c r="F94" s="13"/>
-      <c r="G94" s="13"/>
-      <c r="H94" s="13"/>
-      <c r="I94" s="13"/>
-      <c r="J94" s="13"/>
-      <c r="K94" s="14"/>
-    </row>
-    <row r="95" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B95" s="12"/>
-      <c r="C95" s="13"/>
-      <c r="D95" s="13"/>
-      <c r="E95" s="13"/>
-      <c r="F95" s="13"/>
-      <c r="G95" s="13"/>
-      <c r="H95" s="13"/>
-      <c r="I95" s="13"/>
-      <c r="J95" s="13"/>
-      <c r="K95" s="14"/>
-    </row>
-    <row r="96" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B96" s="12"/>
-      <c r="C96" s="13"/>
-      <c r="D96" s="13"/>
-      <c r="E96" s="13"/>
-      <c r="F96" s="13"/>
-      <c r="G96" s="13"/>
-      <c r="H96" s="13"/>
-      <c r="I96" s="13"/>
-      <c r="J96" s="13"/>
-      <c r="K96" s="14"/>
+      <c r="C89" s="9"/>
+      <c r="D89" s="9"/>
+      <c r="E89" s="9"/>
+      <c r="F89" s="9"/>
+      <c r="G89" s="9"/>
+      <c r="H89" s="9"/>
+      <c r="I89" s="9"/>
+      <c r="J89" s="9"/>
+      <c r="K89" s="10"/>
+    </row>
+    <row r="90" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B90" s="11"/>
+      <c r="K90" s="12"/>
+    </row>
+    <row r="91" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B91" s="11"/>
+      <c r="K91" s="12"/>
+    </row>
+    <row r="92" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B92" s="11"/>
+      <c r="K92" s="12"/>
+    </row>
+    <row r="93" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B93" s="11"/>
+      <c r="K93" s="12"/>
+    </row>
+    <row r="94" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B94" s="11"/>
+      <c r="K94" s="12"/>
+    </row>
+    <row r="95" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B95" s="11"/>
+      <c r="K95" s="12"/>
+    </row>
+    <row r="96" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B96" s="11"/>
+      <c r="K96" s="12"/>
     </row>
     <row r="97" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B97" s="12"/>
-      <c r="C97" s="13"/>
-      <c r="D97" s="13"/>
-      <c r="E97" s="13"/>
-      <c r="F97" s="13"/>
-      <c r="G97" s="13"/>
-      <c r="H97" s="13"/>
-      <c r="I97" s="13"/>
-      <c r="J97" s="13"/>
-      <c r="K97" s="14"/>
+      <c r="B97" s="11"/>
+      <c r="K97" s="12"/>
     </row>
     <row r="98" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B98" s="12"/>
-      <c r="C98" s="13"/>
-      <c r="D98" s="13"/>
-      <c r="E98" s="13"/>
-      <c r="F98" s="13"/>
-      <c r="G98" s="13"/>
-      <c r="H98" s="13"/>
-      <c r="I98" s="13"/>
-      <c r="J98" s="13"/>
-      <c r="K98" s="14"/>
+      <c r="B98" s="11"/>
+      <c r="K98" s="12"/>
     </row>
     <row r="99" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B99" s="12"/>
-      <c r="C99" s="13"/>
-      <c r="D99" s="13"/>
-      <c r="E99" s="13"/>
-      <c r="F99" s="13"/>
-      <c r="G99" s="13"/>
-      <c r="H99" s="13"/>
-      <c r="I99" s="13"/>
-      <c r="J99" s="13"/>
-      <c r="K99" s="14"/>
+      <c r="B99" s="11"/>
+      <c r="K99" s="12"/>
     </row>
     <row r="100" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B100" s="12"/>
-      <c r="C100" s="13"/>
-      <c r="D100" s="13"/>
-      <c r="E100" s="13"/>
-      <c r="F100" s="13"/>
-      <c r="G100" s="13"/>
-      <c r="H100" s="13"/>
-      <c r="I100" s="13"/>
-      <c r="J100" s="13"/>
-      <c r="K100" s="14"/>
+      <c r="B100" s="11"/>
+      <c r="K100" s="12"/>
     </row>
     <row r="101" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B101" s="12"/>
-      <c r="C101" s="13"/>
-      <c r="D101" s="13"/>
-      <c r="E101" s="13"/>
-      <c r="F101" s="13"/>
-      <c r="G101" s="13"/>
-      <c r="H101" s="13"/>
-      <c r="I101" s="13"/>
-      <c r="J101" s="13"/>
-      <c r="K101" s="14"/>
+      <c r="B101" s="11"/>
+      <c r="K101" s="12"/>
     </row>
     <row r="102" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B102" s="12"/>
-      <c r="C102" s="13"/>
-      <c r="D102" s="13"/>
-      <c r="E102" s="13"/>
-      <c r="F102" s="13"/>
-      <c r="G102" s="13"/>
-      <c r="H102" s="13"/>
-      <c r="I102" s="13"/>
-      <c r="J102" s="13"/>
-      <c r="K102" s="14"/>
+      <c r="B102" s="11"/>
+      <c r="K102" s="12"/>
     </row>
     <row r="103" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B103" s="12"/>
-      <c r="C103" s="13"/>
-      <c r="D103" s="13"/>
-      <c r="E103" s="13"/>
-      <c r="F103" s="13"/>
-      <c r="G103" s="13"/>
-      <c r="H103" s="13"/>
-      <c r="I103" s="13"/>
-      <c r="J103" s="13"/>
-      <c r="K103" s="14"/>
+      <c r="B103" s="11"/>
+      <c r="K103" s="12"/>
     </row>
     <row r="104" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B104" s="12"/>
-      <c r="C104" s="13"/>
-      <c r="D104" s="13"/>
-      <c r="E104" s="13"/>
-      <c r="F104" s="13"/>
-      <c r="G104" s="13"/>
-      <c r="H104" s="13"/>
-      <c r="I104" s="13"/>
-      <c r="J104" s="13"/>
-      <c r="K104" s="14"/>
+      <c r="B104" s="11"/>
+      <c r="K104" s="12"/>
     </row>
     <row r="105" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B105" s="12"/>
-      <c r="C105" s="13"/>
-      <c r="D105" s="13"/>
-      <c r="E105" s="13"/>
-      <c r="F105" s="13"/>
-      <c r="G105" s="13"/>
-      <c r="H105" s="13"/>
-      <c r="I105" s="13"/>
-      <c r="J105" s="13"/>
-      <c r="K105" s="14"/>
+      <c r="B105" s="11"/>
+      <c r="K105" s="12"/>
     </row>
     <row r="106" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B106" s="12"/>
-      <c r="C106" s="13"/>
-      <c r="D106" s="13"/>
-      <c r="E106" s="13"/>
-      <c r="F106" s="13"/>
-      <c r="G106" s="13"/>
-      <c r="H106" s="13"/>
-      <c r="I106" s="13"/>
-      <c r="J106" s="13"/>
-      <c r="K106" s="14"/>
+      <c r="B106" s="11"/>
+      <c r="K106" s="12"/>
     </row>
     <row r="107" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B107" s="12"/>
-      <c r="C107" s="13"/>
-      <c r="D107" s="13"/>
-      <c r="E107" s="13"/>
-      <c r="F107" s="13"/>
-      <c r="G107" s="13"/>
-      <c r="H107" s="13"/>
-      <c r="I107" s="13"/>
-      <c r="J107" s="13"/>
-      <c r="K107" s="14"/>
+      <c r="B107" s="11"/>
+      <c r="K107" s="12"/>
     </row>
     <row r="108" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B108" s="12"/>
-      <c r="C108" s="13"/>
-      <c r="D108" s="13"/>
-      <c r="E108" s="13"/>
-      <c r="F108" s="13"/>
-      <c r="G108" s="13"/>
-      <c r="H108" s="13"/>
-      <c r="I108" s="13"/>
-      <c r="J108" s="13"/>
-      <c r="K108" s="14"/>
+      <c r="B108" s="11"/>
+      <c r="K108" s="12"/>
     </row>
     <row r="109" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B109" s="15"/>
-      <c r="C109" s="16"/>
-      <c r="D109" s="16"/>
-      <c r="E109" s="16"/>
-      <c r="F109" s="16"/>
-      <c r="G109" s="16"/>
-      <c r="H109" s="16"/>
-      <c r="I109" s="16"/>
-      <c r="J109" s="16"/>
-      <c r="K109" s="17"/>
+      <c r="B109" s="13"/>
+      <c r="C109" s="14"/>
+      <c r="D109" s="14"/>
+      <c r="E109" s="14"/>
+      <c r="F109" s="14"/>
+      <c r="G109" s="14"/>
+      <c r="H109" s="14"/>
+      <c r="I109" s="14"/>
+      <c r="J109" s="14"/>
+      <c r="K109" s="15"/>
     </row>
     <row r="113" spans="2:2" ht="21" x14ac:dyDescent="0.35">
-      <c r="B113" s="21" t="s">
+      <c r="B113" s="19" t="s">
         <v>226</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="L62:L88">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="greaterThan">
-      <formula>0</formula>
+  <conditionalFormatting sqref="G62:L88">
+    <cfRule type="expression" dxfId="3" priority="6">
+      <formula>$H62="West Sussex"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H59">
-    <cfRule type="expression" dxfId="1" priority="5">
+    <cfRule type="expression" dxfId="2" priority="5">
       <formula>$H62="West Sussex"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G62:L88">
-    <cfRule type="expression" dxfId="0" priority="6">
-      <formula>$H62="West Sussex"</formula>
+  <conditionalFormatting sqref="L62:L88">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="greaterThan">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations disablePrompts="1" count="1">
@@ -10434,7 +10649,7 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" t="s">
         <v>212</v>
       </c>
       <c r="B2">
@@ -10442,7 +10657,7 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="A3" t="s">
         <v>213</v>
       </c>
       <c r="B3">
@@ -10450,7 +10665,7 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="A4" t="s">
         <v>214</v>
       </c>
       <c r="B4">
@@ -10458,7 +10673,7 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="A5" t="s">
         <v>215</v>
       </c>
       <c r="B5">
@@ -10466,7 +10681,7 @@
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" t="s">
         <v>216</v>
       </c>
       <c r="B6">

</xml_diff>